<commit_message>
Actualizacion automatica de datos - mar 04/08/2026 19:28:58,63
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Agosto.xlsx
+++ b/Cronograma de Tareas/Cronograma Agosto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{555101DE-3D4C-4AE8-864B-824681CAE292}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{98BEDEB8-80D0-4DE0-A56F-770C1F3168B7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{98BEDEB8-80D0-4DE0-A56F-770C1F3168B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 3 al 9 Ago" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="94">
   <si>
     <t>Set 1 Mañana</t>
   </si>
@@ -326,9 +326,6 @@
     <t>Respuesta Contracargos (Correo) desde las 6:00 pm</t>
   </si>
   <si>
-    <t xml:space="preserve">Josue </t>
-  </si>
-  <si>
     <t xml:space="preserve">Alejandra </t>
   </si>
   <si>
@@ -348,6 +345,9 @@
   </si>
   <si>
     <t>Respuesta Contracargos (Correo) desde las 11:00 am</t>
+  </si>
+  <si>
+    <t>Juan Jose / Oriana</t>
   </si>
 </sst>
 </file>
@@ -491,11 +491,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -543,29 +540,674 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="65">
+  <dxfs count="131">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1547,906 +2189,915 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB30B516-10BE-4D09-A029-062BDDADE196}">
   <dimension ref="B2:L41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="62.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7" style="3" customWidth="1"/>
-    <col min="5" max="5" width="62.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.85546875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="52.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.42578125" style="3" customWidth="1"/>
-    <col min="11" max="11" width="54" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="15" style="3"/>
+    <col min="1" max="1" width="3.44140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="51.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" style="2" customWidth="1"/>
+    <col min="5" max="5" width="56.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.88671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="46.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.44140625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="48.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="15" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B2" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="1" t="s">
+      <c r="C2" s="18"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="1"/>
-      <c r="H2" s="1" t="s">
+      <c r="F2" s="18"/>
+      <c r="H2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="1"/>
-      <c r="K2" s="1" t="s">
+      <c r="I2" s="18"/>
+      <c r="K2" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="L2" s="1"/>
-    </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B3" s="4" t="s">
+      <c r="L2" s="18"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="4" t="s">
+      <c r="D3" s="1"/>
+      <c r="E3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="L3" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="5" t="s">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K4" s="7" t="s">
+      <c r="K4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L4" s="8" t="s">
+      <c r="L4" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="7" t="s">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="I5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="19" t="s">
+      <c r="K5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="L5" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="7" t="s">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="I6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K6" s="19" t="s">
+      <c r="K6" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="L6" s="20" t="s">
+      <c r="L6" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="7" t="s">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B7" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="I7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="K7" s="21" t="s">
+      <c r="K7" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="L7" s="20" t="s">
+      <c r="L7" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="7" t="s">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B8" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K8" s="22" t="s">
+      <c r="K8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="L8" s="20" t="s">
+      <c r="L8" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="7" t="s">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B9" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="I9" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="K9" s="19" t="s">
+      <c r="K9" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="L9" s="20" t="s">
+      <c r="L9" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="7" t="s">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B10" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="I10" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K10" s="19" t="s">
+      <c r="K10" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L10" s="20" t="s">
+      <c r="L10" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="E11" s="7" t="s">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="E11" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="I11" s="8" t="s">
+      <c r="I11" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="K11" s="19" t="s">
+      <c r="K11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="L11" s="20" t="s">
+      <c r="L11" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="1" t="s">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B12" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="H12" s="7" t="s">
+      <c r="C12" s="18"/>
+      <c r="H12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="8" t="s">
+      <c r="I12" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K12" s="19" t="s">
+      <c r="K12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="L12" s="20" t="s">
+      <c r="L12" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="4" t="s">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B13" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="1" t="s">
+      <c r="D13" s="1"/>
+      <c r="E13" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="F13" s="1"/>
-      <c r="H13" s="7" t="s">
+      <c r="F13" s="18"/>
+      <c r="H13" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I13" s="8" t="s">
+      <c r="I13" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="K13" s="19" t="s">
+      <c r="K13" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="L13" s="20" t="s">
+      <c r="L13" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B14" s="7" t="s">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B14" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="4" t="s">
+      <c r="D14" s="1"/>
+      <c r="E14" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="H14" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="I14" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K14" s="23" t="s">
+      <c r="K14" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="L14" s="20" t="s">
+      <c r="L14" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B15" s="7" t="s">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B15" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H15" s="10" t="s">
+      <c r="H15" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="I15" s="8" t="s">
+      <c r="I15" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="K15" s="24" t="s">
+      <c r="K15" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="L15" s="20" t="s">
+      <c r="L15" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B16" s="7" t="s">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B16" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G16" s="2"/>
-      <c r="J16" s="2"/>
-    </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B17" s="7" t="s">
+      <c r="G16" s="1"/>
+      <c r="J16" s="1"/>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B17" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H17" s="1" t="s">
+      <c r="H17" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="I17" s="1"/>
-      <c r="K17" s="1" t="s">
+      <c r="I17" s="18"/>
+      <c r="K17" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="L17" s="1"/>
-    </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B18" s="9" t="s">
+      <c r="L17" s="18"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B18" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="E18" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="F18" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="H18" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="I18" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="K18" s="4" t="s">
+      <c r="K18" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="L18" s="13" t="s">
+      <c r="L18" s="12" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="12" t="s">
+    <row r="19" spans="2:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H19" s="7" t="s">
+      <c r="H19" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I19" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="K19" s="14" t="s">
+      <c r="I19" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K19" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="L19" s="6" t="s">
+      <c r="L19" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="9" t="s">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B20" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="15" t="s">
+      <c r="E20" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="F20" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="H20" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="I20" s="6" t="s">
+      <c r="I20" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="K20" s="14" t="s">
+      <c r="K20" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="L20" s="6" t="s">
+      <c r="L20" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B21" s="7" t="s">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B21" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H21" s="5" t="s">
+      <c r="H21" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I21" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="K21" s="14" t="s">
+      <c r="I21" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K21" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="L21" s="6" t="s">
+      <c r="L21" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B22" s="7" t="s">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B22" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H22" s="7" t="s">
+      <c r="E22" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F22" s="18"/>
+      <c r="H22" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="I22" s="6" t="s">
+      <c r="I22" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="K22" s="14" t="s">
+      <c r="K22" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="L22" s="6" t="s">
+      <c r="L22" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="E23" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F23" s="1"/>
-      <c r="H23" s="7" t="s">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="E23" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H23" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="I23" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="K23" s="14" t="s">
+      <c r="I23" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K23" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="L23" s="6" t="s">
+      <c r="L23" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B24" s="1" t="s">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B24" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="C24" s="1"/>
-      <c r="E24" s="4" t="s">
+      <c r="C24" s="18"/>
+      <c r="E24" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K24" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="L24" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B25" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K25" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="L25" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B26" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K26" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="L26" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B27" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K27" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="L27" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B28" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H28" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K28" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="L28" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B29" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B30" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="H30" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="I30" s="18"/>
+      <c r="K30" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="L30" s="18"/>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="H31" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="I31" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H24" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I24" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="K24" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="L24" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B25" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C25" s="4" t="s">
+      <c r="K31" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="L31" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E25" s="7" t="s">
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="D32"/>
+      <c r="H32" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F25" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="I25" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="K25" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="L25" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B26" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E26" s="7" t="s">
+      <c r="I32" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L32" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="D33"/>
+      <c r="H33" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H26" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I26" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="K26" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="L26" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B27" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H27" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="I27" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="K27" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="L27" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B28" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H28" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="I28" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="K28" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="L28" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B29"/>
-      <c r="C29"/>
-      <c r="E29" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="H30" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I30" s="1"/>
-      <c r="K30" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L30" s="1"/>
-    </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="H31" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="I31" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="K31" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="L31" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="D32"/>
-      <c r="H32" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I32" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K32" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="L32" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="D33"/>
-      <c r="H33" s="7" t="s">
+      <c r="I33" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K33" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="I33" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K33" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="L33" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L33" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34"/>
       <c r="C34"/>
       <c r="D34"/>
-      <c r="H34" s="7" t="s">
+      <c r="H34" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I34" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K34" s="7" t="s">
+      <c r="I34" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K34" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="L34" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L34" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D35"/>
-      <c r="H35" s="7" t="s">
+      <c r="H35" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="I35" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K35" s="7" t="s">
+      <c r="I35" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K35" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="L35" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L35" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D36"/>
-      <c r="H36" s="7" t="s">
+      <c r="H36" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="I36" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K36" s="7" t="s">
+      <c r="I36" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K36" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="L36" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L36" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D37"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D38"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D39"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D40"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D41"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="aL/0A1WcO5wh8HIUN2M4OdxiD0qUWblDC3AbV+wgqpgBsV61JCOeN7urSAxfZTI1Oq/QMb5clSyvytBtW5lOWQ==" saltValue="TUcYVmGU0hlw2l7ddYgNpA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B24:C24"/>
-    <mergeCell ref="E23:F23"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E13:F13"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="E13:F13"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="64" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="63" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="62" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="24"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B21">
+    <cfRule type="duplicateValues" dxfId="61" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B26 E17:E18 B20">
+    <cfRule type="duplicateValues" dxfId="60" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27 B9">
-    <cfRule type="duplicateValues" dxfId="61" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="32"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6">
+    <cfRule type="duplicateValues" dxfId="58" priority="23"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7">
+    <cfRule type="duplicateValues" dxfId="57" priority="22"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E8">
+    <cfRule type="duplicateValues" dxfId="56" priority="21"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9">
+    <cfRule type="duplicateValues" dxfId="55" priority="26"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E10">
+    <cfRule type="duplicateValues" dxfId="54" priority="16"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E11">
+    <cfRule type="duplicateValues" dxfId="53" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E19 B10">
-    <cfRule type="duplicateValues" dxfId="60" priority="33"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B26 E17:E18 B20">
-    <cfRule type="duplicateValues" dxfId="59" priority="34"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B21">
-    <cfRule type="duplicateValues" dxfId="58" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="57" priority="26"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="56" priority="25"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="55" priority="24"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="54" priority="29"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E10">
-    <cfRule type="duplicateValues" dxfId="53" priority="19"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E11">
-    <cfRule type="duplicateValues" dxfId="52" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="30"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E27">
+    <cfRule type="duplicateValues" dxfId="51" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E28">
-    <cfRule type="duplicateValues" dxfId="51" priority="17"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E29">
-    <cfRule type="duplicateValues" dxfId="50" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="49" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="48" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="47" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="46" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="45" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="44" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="43" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="42" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="41" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="40" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="39" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="38" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="37" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="28"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K23">
+    <cfRule type="duplicateValues" dxfId="36" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24:K25">
-    <cfRule type="duplicateValues" dxfId="36" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="35" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="34" priority="7"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K23">
-    <cfRule type="duplicateValues" dxfId="33" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="5"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2455,817 +3106,811 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBD94355-E31A-4000-9852-300E7332D394}">
   <dimension ref="B2:L41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="62.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7" style="3" customWidth="1"/>
-    <col min="5" max="5" width="52.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.85546875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="52.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.42578125" style="3" customWidth="1"/>
-    <col min="11" max="11" width="54" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="15" style="3"/>
+    <col min="1" max="1" width="3.44140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="56.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" style="2" customWidth="1"/>
+    <col min="5" max="5" width="46.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6" style="2" customWidth="1"/>
+    <col min="8" max="8" width="49.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.44140625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="54" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="15" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B2" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="1" t="s">
+      <c r="C2" s="18"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="1"/>
-      <c r="H2" s="1" t="s">
+      <c r="F2" s="18"/>
+      <c r="H2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="1"/>
-      <c r="K2" s="1" t="s">
+      <c r="I2" s="18"/>
+      <c r="K2" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="L2" s="1"/>
-    </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B3" s="4" t="s">
+      <c r="L2" s="18"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="4" t="s">
+      <c r="D3" s="1"/>
+      <c r="E3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="L3" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="5" t="s">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="K4" s="7" t="s">
+      <c r="I5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L4" s="8" t="s">
+      <c r="C6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L6" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="6" t="s">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="6" t="s">
+      <c r="E7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="I5" s="8" t="s">
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B9" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="I9" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="K5" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="L5" s="20" t="s">
+      <c r="K9" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B10" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="E11" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="F11" s="18"/>
+      <c r="H11" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B12" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="18"/>
+      <c r="E12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B13" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B14" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="K14" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B15" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="K15" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B16" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" s="1"/>
+      <c r="J16" s="1"/>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B17" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H17" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="I17" s="18"/>
+      <c r="K17" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="L17" s="18"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B18" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="L18" s="12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K19" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="L19" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="E20" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F20" s="18"/>
+      <c r="H20" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K20" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="L20" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B21" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" s="18"/>
+      <c r="E21" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H21" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K21" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="L21" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B22" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H22" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I22" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K22" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="L22" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B23" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="6" t="s">
+      <c r="E23" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H23" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K23" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="L23" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="L6" s="20" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="7" t="s">
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B24" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H24" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K24" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="L24" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B25" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H25" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="I7" s="8" t="s">
+      <c r="I25" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K25" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="L25" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B26" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K26" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="L26" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B27" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H27" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K27" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="L27" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B28" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H28" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K28" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="L28" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B29" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="K7" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="L7" s="20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="L8" s="20" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="I9" s="8" t="s">
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B30" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C30" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="K9" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="L9" s="20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="I10" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="K10" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="L10" s="20" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="E11" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F11" s="1"/>
-      <c r="H11" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="I11" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="K11" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="L11" s="20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="1"/>
-      <c r="E12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F12" s="4" t="s">
+      <c r="H30" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="I30" s="18"/>
+      <c r="K30" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="L30" s="18"/>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B31" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I31" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H12" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="K12" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="L12" s="20" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" s="4" t="s">
+      <c r="K31" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="L31" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="7" t="s">
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B32" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D32"/>
+      <c r="H32" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F13" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="I13" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="K13" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="L13" s="20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B14" s="7" t="s">
+      <c r="I32" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K32" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H14" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="I14" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="K14" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="L14" s="20" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B15" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="K15" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="L15" s="20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B16" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="G16" s="2"/>
-      <c r="J16" s="2"/>
-    </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B17" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I17" s="1"/>
-      <c r="K17" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="L17" s="1"/>
-    </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B18" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="K18" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="L18" s="13" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H19" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="I19" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K19" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="L19" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="H20" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I20" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K20" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="L20" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B21" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C21" s="1"/>
-      <c r="E21" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F21" s="1"/>
-      <c r="H21" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="I21" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K21" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="L21" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B22" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H22" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="I22" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K22" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="L22" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B23" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F23" s="6" t="s">
+      <c r="L32" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H23" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="I23" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K23" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="L23" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B24" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="I24" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K24" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="L24" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B25" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="H25" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="I25" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K25" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="L25" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B26" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E26" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="H26" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="I26" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K26" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="L26" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B27" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="H27" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="I27" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K27" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="L27" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B28" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H28" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="I28" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K28" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="L28" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B29" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B30" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I30" s="1"/>
-      <c r="K30" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L30" s="1"/>
-    </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B31" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="H31" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="I31" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="K31" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="L31" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B32" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D32"/>
-      <c r="H32" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I32" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K32" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="L32" s="6" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33"/>
       <c r="C33"/>
       <c r="D33"/>
-      <c r="H33" s="7" t="s">
+      <c r="H33" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="I33" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K33" s="7" t="s">
+      <c r="I33" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K33" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="L33" s="6" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L33" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34"/>
       <c r="C34"/>
       <c r="D34"/>
-      <c r="H34" s="7" t="s">
+      <c r="H34" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I34" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K34" s="7" t="s">
+      <c r="I34" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K34" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="L34" s="6" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L34" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35"/>
       <c r="C35"/>
       <c r="D35"/>
-      <c r="H35" s="7" t="s">
+      <c r="H35" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="I35" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K35" s="7" t="s">
+      <c r="I35" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K35" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="L35" s="6" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L35" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D36"/>
-      <c r="H36" s="7" t="s">
+      <c r="H36" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="I36" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K36" s="7" t="s">
+      <c r="I36" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K36" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="L36" s="6" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L36" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D37"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D38"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D39"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D40"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="D41"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="+TX5riWQ6famA0LHqLZB9jh+Ubt81EZBktEHoUNWLTB07fl8KTMX0K8LEf+TJkGHpe4VgLXWd//1JYTA9plGXA==" saltValue="KY4N8o/BWNEpQJFrrrdORw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
@@ -3273,105 +3918,110 @@
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E20:F20"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="32" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="31" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="30" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="26"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B23:B25">
+    <cfRule type="duplicateValues" dxfId="29" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26 B9">
-    <cfRule type="duplicateValues" dxfId="29" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27 B10">
-    <cfRule type="duplicateValues" dxfId="28" priority="39"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B23:B25">
-    <cfRule type="duplicateValues" dxfId="27" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="31"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B30">
+    <cfRule type="duplicateValues" dxfId="26" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B32">
+    <cfRule type="duplicateValues" dxfId="25" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="26" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="25" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="24" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="23" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16">
-    <cfRule type="duplicateValues" dxfId="22" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="21" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E18">
+    <cfRule type="duplicateValues" dxfId="18" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E25">
+    <cfRule type="duplicateValues" dxfId="17" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26">
-    <cfRule type="duplicateValues" dxfId="20" priority="23"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E27">
-    <cfRule type="duplicateValues" dxfId="19" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="18" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="17" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="16" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="15" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="29"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H23">
+    <cfRule type="duplicateValues" dxfId="11" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H24:H25">
+    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="14" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="13" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4">
+    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11">
+    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12">
+    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K13">
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K23">
+    <cfRule type="duplicateValues" dxfId="3" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24:K25">
-    <cfRule type="duplicateValues" dxfId="12" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="11" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="10" priority="14"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K23">
-    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B30">
-    <cfRule type="duplicateValues" dxfId="8" priority="9"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B32">
-    <cfRule type="duplicateValues" dxfId="7" priority="8"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E18">
-    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H24:H25">
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H23">
-    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="12"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3380,209 +4030,209 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B623CE4C-92BF-4BB6-8978-4FC3B181F198}">
   <dimension ref="A1:B25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="95.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="95.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="47.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="94.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="94.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="15" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="8" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+    <row r="4" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="8" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+    <row r="5" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="8" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+    <row r="6" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="8" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="17" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
+    <row r="8" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="8" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
+    <row r="9" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="8" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
+    <row r="11" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="8" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="17" t="s">
+    <row r="12" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="8" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="17" t="s">
+    <row r="13" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="8" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
+    <row r="14" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="8" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="135" x14ac:dyDescent="0.25">
-      <c r="A15" s="17" t="s">
+    <row r="15" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="8" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="105" x14ac:dyDescent="0.25">
-      <c r="A16" s="17" t="s">
+    <row r="16" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="8" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A17" s="17" t="s">
+    <row r="17" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="8" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="17" t="s">
+    <row r="18" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="8" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="17" t="s">
+    <row r="19" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="8" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="150" x14ac:dyDescent="0.25">
-      <c r="A20" s="17" t="s">
+    <row r="20" spans="1:2" ht="144" x14ac:dyDescent="0.3">
+      <c r="A20" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A21" s="17" t="s">
+    <row r="21" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="8" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A22" s="18" t="s">
+    <row r="22" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A22" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="8" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="105" x14ac:dyDescent="0.25">
-      <c r="A23" s="17" t="s">
+    <row r="23" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="8" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A24" s="17" t="s">
+    <row r="24" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="8" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A25" s="17" t="s">
+    <row r="25" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="8" t="s">
         <v>79</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion automatica de datos - jue 06/08/2026 10:49:21,96
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Agosto.xlsx
+++ b/Cronograma de Tareas/Cronograma Agosto.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{555101DE-3D4C-4AE8-864B-824681CAE292}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C0992CE-E419-4875-A3E9-9559EB56EAC3}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{98BEDEB8-80D0-4DE0-A56F-770C1F3168B7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{98BEDEB8-80D0-4DE0-A56F-770C1F3168B7}"/>
   </bookViews>
   <sheets>
-    <sheet name="Semana 1 - 3 al 9 Ago" sheetId="1" r:id="rId1"/>
-    <sheet name="Semana 2 - 10 al 16 Ago" sheetId="3" r:id="rId2"/>
+    <sheet name="Semana 1 - 3 al 9 Ago" sheetId="4" r:id="rId1"/>
+    <sheet name="Semana 2 - 10 al 16 Ago" sheetId="5" r:id="rId2"/>
     <sheet name="Detalle Cronograma" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -547,667 +547,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="131">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="65">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2187,7 +1527,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB30B516-10BE-4D09-A029-062BDDADE196}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE1A42CC-46E2-451F-A6D1-C9AFFEA79DB3}">
   <dimension ref="B2:L41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2989,19 +2329,20 @@
       <c r="D41"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="IUqCyFrkbaZZs6cAzVH6yADvOKVmD+jfZ62LKfyUlQEBibwLjteZyT+2HPzW7vehSpQu4vmXZgLgmCKrwS2vqg==" saltValue="mjSDMFqxFcyaLmjD30rnTw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E22:F22"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="E13:F13"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B12:C12"/>
+    <mergeCell ref="E13:F13"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="64" priority="29"/>
@@ -3104,7 +2445,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBD94355-E31A-4000-9852-300E7332D394}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{915BA1CC-8A13-44B5-B15A-B30897755693}">
   <dimension ref="B2:L41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3910,7 +3251,12 @@
       <c r="D41"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="oIouQdWR80zfwrOgYg8mubgJdhcsB76Q9F8KDvzgM4ZHVaoaTdmBWqCttJGfgtEQSU1Z0+MmOBTlntxS+E5R6w==" saltValue="noKwfl3/0vFaNfkmv2IeLw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="B21:C21"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
@@ -3919,10 +3265,6 @@
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="E20:F20"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="32" priority="30"/>

</xml_diff>

<commit_message>
Actualizacion automatica de datos - vie 14/08/2026 14:20:45,42
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Agosto.xlsx
+++ b/Cronograma de Tareas/Cronograma Agosto.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C0992CE-E419-4875-A3E9-9559EB56EAC3}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B64BFF3-983D-4702-AD2B-0199540AD160}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{98BEDEB8-80D0-4DE0-A56F-770C1F3168B7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{98BEDEB8-80D0-4DE0-A56F-770C1F3168B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 3 al 9 Ago" sheetId="4" r:id="rId1"/>
     <sheet name="Semana 2 - 10 al 16 Ago" sheetId="5" r:id="rId2"/>
-    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId3"/>
+    <sheet name="Semana 3 - 17 al 23 Ago" sheetId="6" r:id="rId3"/>
+    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="98">
   <si>
     <t>Set 1 Mañana</t>
   </si>
@@ -348,6 +349,18 @@
   </si>
   <si>
     <t>Juan Jose / Oriana</t>
+  </si>
+  <si>
+    <t>Alerta SEON (Correo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Josue </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yefferson </t>
+  </si>
+  <si>
+    <t>Revisión Calendarios</t>
   </si>
 </sst>
 </file>
@@ -491,7 +504,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -543,11 +556,394 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="65">
+  <dxfs count="103">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1529,24 +1925,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE1A42CC-46E2-451F-A6D1-C9AFFEA79DB3}">
   <dimension ref="B2:L41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.44140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="51.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="51.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7" style="2" customWidth="1"/>
-    <col min="5" max="5" width="56.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.88671875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="46.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="56.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.85546875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="46.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.44140625" style="2" customWidth="1"/>
-    <col min="11" max="11" width="48.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.42578125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="48.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="15" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" s="18" t="s">
         <v>0</v>
       </c>
@@ -1565,7 +1961,7 @@
       </c>
       <c r="L2" s="18"/>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1592,7 +1988,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
@@ -1618,7 +2014,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
         <v>13</v>
       </c>
@@ -1644,7 +2040,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
         <v>10</v>
       </c>
@@ -1670,7 +2066,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
         <v>18</v>
       </c>
@@ -1696,7 +2092,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
         <v>20</v>
       </c>
@@ -1722,7 +2118,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
         <v>23</v>
       </c>
@@ -1748,7 +2144,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
         <v>31</v>
       </c>
@@ -1774,7 +2170,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="E11" s="6" t="s">
         <v>31</v>
       </c>
@@ -1794,7 +2190,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="18" t="s">
         <v>26</v>
       </c>
@@ -1812,7 +2208,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
         <v>4</v>
       </c>
@@ -1837,7 +2233,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="6" t="s">
         <v>16</v>
       </c>
@@ -1864,7 +2260,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
         <v>19</v>
       </c>
@@ -1890,7 +2286,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="6" t="s">
         <v>24</v>
       </c>
@@ -1906,7 +2302,7 @@
       <c r="G16" s="1"/>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="6" t="s">
         <v>32</v>
       </c>
@@ -1928,7 +2324,7 @@
       </c>
       <c r="L17" s="18"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
         <v>21</v>
       </c>
@@ -1954,7 +2350,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="2:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="11" t="s">
         <v>33</v>
       </c>
@@ -1980,7 +2376,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="8" t="s">
         <v>47</v>
       </c>
@@ -2006,7 +2402,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="6" t="s">
         <v>48</v>
       </c>
@@ -2026,7 +2422,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="6" t="s">
         <v>80</v>
       </c>
@@ -2050,7 +2446,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="E23" s="3" t="s">
         <v>40</v>
       </c>
@@ -2070,7 +2466,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="18" t="s">
         <v>37</v>
       </c>
@@ -2094,7 +2490,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="3" t="s">
         <v>4</v>
       </c>
@@ -2120,7 +2516,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="8" t="s">
         <v>43</v>
       </c>
@@ -2146,7 +2542,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="6" t="s">
         <v>45</v>
       </c>
@@ -2172,7 +2568,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="6" t="s">
         <v>36</v>
       </c>
@@ -2198,7 +2594,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="14" t="s">
         <v>29</v>
       </c>
@@ -2206,7 +2602,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="6" t="s">
         <v>41</v>
       </c>
@@ -2222,7 +2618,7 @@
       </c>
       <c r="L30" s="18"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H31" s="3" t="s">
         <v>40</v>
       </c>
@@ -2236,7 +2632,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D32"/>
       <c r="H32" s="6" t="s">
         <v>16</v>
@@ -2251,7 +2647,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D33"/>
       <c r="H33" s="6" t="s">
         <v>19</v>
@@ -2266,7 +2662,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34"/>
       <c r="C34"/>
       <c r="D34"/>
@@ -2283,7 +2679,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D35"/>
       <c r="H35" s="6" t="s">
         <v>29</v>
@@ -2298,7 +2694,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D36"/>
       <c r="H36" s="6" t="s">
         <v>31</v>
@@ -2313,132 +2709,132 @@
         <v>28</v>
       </c>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D37"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D38"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D39"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D40"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D41"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="IUqCyFrkbaZZs6cAzVH6yADvOKVmD+jfZ62LKfyUlQEBibwLjteZyT+2HPzW7vehSpQu4vmXZgLgmCKrwS2vqg==" saltValue="mjSDMFqxFcyaLmjD30rnTw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B12:C12"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="E13:F13"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="64" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="102" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="63" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="101" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="62" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21">
-    <cfRule type="duplicateValues" dxfId="61" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="99" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26 E17:E18 B20">
-    <cfRule type="duplicateValues" dxfId="60" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="98" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27 B9">
-    <cfRule type="duplicateValues" dxfId="59" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="58" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="57" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="56" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="55" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10">
-    <cfRule type="duplicateValues" dxfId="54" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11">
-    <cfRule type="duplicateValues" dxfId="53" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E19 B10">
-    <cfRule type="duplicateValues" dxfId="52" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E27">
-    <cfRule type="duplicateValues" dxfId="51" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E28">
-    <cfRule type="duplicateValues" dxfId="50" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="49" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="48" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="47" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="46" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="45" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="44" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="43" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="42" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="41" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="40" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="39" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="38" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="37" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K23">
-    <cfRule type="duplicateValues" dxfId="36" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24:K25">
-    <cfRule type="duplicateValues" dxfId="35" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="34" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="33" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="5"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2447,24 +2843,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{915BA1CC-8A13-44B5-B15A-B30897755693}">
   <dimension ref="B2:L41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.44140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="56.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="56.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7" style="2" customWidth="1"/>
-    <col min="5" max="5" width="46.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="46.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6" style="2" customWidth="1"/>
-    <col min="8" max="8" width="49.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.44140625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="49.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.42578125" style="2" customWidth="1"/>
     <col min="11" max="11" width="54" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="15" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" s="18" t="s">
         <v>0</v>
       </c>
@@ -2483,7 +2879,7 @@
       </c>
       <c r="L2" s="18"/>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
@@ -2510,7 +2906,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
@@ -2536,7 +2932,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
         <v>13</v>
       </c>
@@ -2562,7 +2958,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
         <v>10</v>
       </c>
@@ -2588,7 +2984,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
         <v>18</v>
       </c>
@@ -2614,7 +3010,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
         <v>20</v>
       </c>
@@ -2640,7 +3036,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
         <v>23</v>
       </c>
@@ -2666,7 +3062,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
         <v>31</v>
       </c>
@@ -2686,7 +3082,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="E11" s="18" t="s">
         <v>1</v>
       </c>
@@ -2704,7 +3100,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="18" t="s">
         <v>26</v>
       </c>
@@ -2728,7 +3124,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
         <v>4</v>
       </c>
@@ -2755,7 +3151,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="6" t="s">
         <v>16</v>
       </c>
@@ -2782,7 +3178,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="6" t="s">
         <v>19</v>
       </c>
@@ -2808,7 +3204,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="6" t="s">
         <v>24</v>
       </c>
@@ -2824,7 +3220,7 @@
       <c r="G16" s="1"/>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="6" t="s">
         <v>32</v>
       </c>
@@ -2846,7 +3242,7 @@
       </c>
       <c r="L17" s="18"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
         <v>21</v>
       </c>
@@ -2872,7 +3268,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="2:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="8" t="s">
         <v>33</v>
       </c>
@@ -2892,7 +3288,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="E20" s="18" t="s">
         <v>38</v>
       </c>
@@ -2910,7 +3306,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="18" t="s">
         <v>37</v>
       </c>
@@ -2934,7 +3330,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="3" t="s">
         <v>4</v>
       </c>
@@ -2960,7 +3356,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="8" t="s">
         <v>39</v>
       </c>
@@ -2986,7 +3382,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
         <v>41</v>
       </c>
@@ -3012,7 +3408,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="8" t="s">
         <v>43</v>
       </c>
@@ -3038,7 +3434,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="6" t="s">
         <v>45</v>
       </c>
@@ -3064,7 +3460,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="6" t="s">
         <v>29</v>
       </c>
@@ -3084,7 +3480,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="14" t="s">
         <v>46</v>
       </c>
@@ -3104,7 +3500,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="6" t="s">
         <v>36</v>
       </c>
@@ -3112,7 +3508,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="6" t="s">
         <v>48</v>
       </c>
@@ -3128,7 +3524,7 @@
       </c>
       <c r="L30" s="18"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="6" t="s">
         <v>80</v>
       </c>
@@ -3148,7 +3544,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="8" t="s">
         <v>47</v>
       </c>
@@ -3169,7 +3565,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33"/>
       <c r="C33"/>
       <c r="D33"/>
@@ -3186,7 +3582,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34"/>
       <c r="C34"/>
       <c r="D34"/>
@@ -3203,7 +3599,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35"/>
       <c r="C35"/>
       <c r="D35"/>
@@ -3220,7 +3616,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D36"/>
       <c r="H36" s="6" t="s">
         <v>31</v>
@@ -3235,150 +3631,1110 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D37"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D38"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D39"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D40"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D41"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="oIouQdWR80zfwrOgYg8mubgJdhcsB76Q9F8KDvzgM4ZHVaoaTdmBWqCttJGfgtEQSU1Z0+MmOBTlntxS+E5R6w==" saltValue="noKwfl3/0vFaNfkmv2IeLw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="B12:C12"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="32" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="31" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="30" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:B25">
-    <cfRule type="duplicateValues" dxfId="29" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26 B9">
-    <cfRule type="duplicateValues" dxfId="28" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27 B10">
-    <cfRule type="duplicateValues" dxfId="27" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
-    <cfRule type="duplicateValues" dxfId="26" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32">
-    <cfRule type="duplicateValues" dxfId="25" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="24" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="23" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="22" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="21" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16">
-    <cfRule type="duplicateValues" dxfId="20" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="19" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18">
-    <cfRule type="duplicateValues" dxfId="18" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
-    <cfRule type="duplicateValues" dxfId="17" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26">
-    <cfRule type="duplicateValues" dxfId="16" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="15" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="14" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="13" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="12" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H23">
-    <cfRule type="duplicateValues" dxfId="11" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24:H25">
-    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="9" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="8" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K23">
-    <cfRule type="duplicateValues" dxfId="3" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24:K25">
-    <cfRule type="duplicateValues" dxfId="2" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="1" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="0" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="12"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFC57F5E-00D1-4280-BD6D-26FE3A9211D7}">
+  <dimension ref="B2:L41"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="3.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="54.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" style="2" customWidth="1"/>
+    <col min="5" max="5" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6" style="2" customWidth="1"/>
+    <col min="8" max="8" width="55" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.42578125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="55" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="15" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="18"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="18"/>
+      <c r="H2" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="I2" s="18"/>
+      <c r="K2" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="L2" s="18"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B9" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B10" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B11" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="E12" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B13" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="18"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="K14" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="K15" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B16" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G16" s="1"/>
+      <c r="H16" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="J16" s="1"/>
+      <c r="K16" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B17" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B18" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18" s="18"/>
+      <c r="H18" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="I18" s="18"/>
+      <c r="K18" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="L18" s="18"/>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B19" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="L19" s="12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="B20" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="H20" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="K20" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="L20" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="E21" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="H21" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K21" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="L21" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B22" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22" s="18"/>
+      <c r="E22" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="H22" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="I22" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="K22" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="L22" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B23" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="H23" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K23" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="L23" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B24" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="H24" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="K24" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="L24" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="B25" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H25" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K25" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="L25" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B26" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="K26" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="L26" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B27" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H27" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K27" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="L27" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H28" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="K28" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="L28" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B29" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H29" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K29" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="L29" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B30" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H30" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="J30" s="1"/>
+      <c r="K30" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="L30" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B31" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B32" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D32"/>
+      <c r="H32" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="I32" s="18"/>
+      <c r="K32" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="L32" s="18"/>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B33" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D33"/>
+      <c r="H33" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K33" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="L33" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D34"/>
+      <c r="H34" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L34" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D35"/>
+      <c r="H35" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L35" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D36"/>
+      <c r="H36" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="L36" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D37"/>
+      <c r="H37" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I37" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L37" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D38"/>
+      <c r="H38" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I38" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="L38" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D39"/>
+    </row>
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D40"/>
+    </row>
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D41"/>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="K18:L18"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="duplicateValues" dxfId="37" priority="35"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7">
+    <cfRule type="duplicateValues" dxfId="36" priority="32"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8">
+    <cfRule type="duplicateValues" dxfId="35" priority="31"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B28 B9">
+    <cfRule type="duplicateValues" dxfId="34" priority="37"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B31 B10">
+    <cfRule type="duplicateValues" dxfId="33" priority="36"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29 B26">
+    <cfRule type="duplicateValues" dxfId="32" priority="13"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6">
+    <cfRule type="duplicateValues" dxfId="31" priority="30"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7">
+    <cfRule type="duplicateValues" dxfId="30" priority="29"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E8">
+    <cfRule type="duplicateValues" dxfId="29" priority="28"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9">
+    <cfRule type="duplicateValues" dxfId="28" priority="33"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E10">
+    <cfRule type="duplicateValues" dxfId="27" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E14">
+    <cfRule type="duplicateValues" dxfId="26" priority="25"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E15">
+    <cfRule type="duplicateValues" dxfId="25" priority="24"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E16">
+    <cfRule type="duplicateValues" dxfId="24" priority="12"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B33">
+    <cfRule type="duplicateValues" dxfId="23" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E23">
+    <cfRule type="duplicateValues" dxfId="22" priority="23"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E24">
+    <cfRule type="duplicateValues" dxfId="21" priority="22"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4">
+    <cfRule type="duplicateValues" dxfId="20" priority="16"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="duplicateValues" dxfId="19" priority="27"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12">
+    <cfRule type="duplicateValues" dxfId="18" priority="26"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="duplicateValues" dxfId="17" priority="34"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H16">
+    <cfRule type="duplicateValues" dxfId="16" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H24">
+    <cfRule type="duplicateValues" dxfId="15" priority="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25:H26">
+    <cfRule type="duplicateValues" dxfId="14" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H30">
+    <cfRule type="duplicateValues" dxfId="13" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H37">
+    <cfRule type="duplicateValues" dxfId="12" priority="20"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H38">
+    <cfRule type="duplicateValues" dxfId="11" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4">
+    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11">
+    <cfRule type="duplicateValues" dxfId="9" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12">
+    <cfRule type="duplicateValues" dxfId="8" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K13">
+    <cfRule type="duplicateValues" dxfId="7" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K16">
+    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K24">
+    <cfRule type="duplicateValues" dxfId="5" priority="15"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K25:K26">
+    <cfRule type="duplicateValues" dxfId="4" priority="21"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K30">
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K37">
+    <cfRule type="duplicateValues" dxfId="2" priority="18"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K38">
+    <cfRule type="duplicateValues" dxfId="1" priority="17"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B27 B24 B11">
+    <cfRule type="duplicateValues" dxfId="0" priority="38"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B623CE4C-92BF-4BB6-8978-4FC3B181F198}">
   <dimension ref="A1:B25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="95.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="95.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="94.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="94.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
         <v>51</v>
       </c>
@@ -3386,7 +4742,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
         <v>13</v>
       </c>
@@ -3394,7 +4750,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
         <v>7</v>
       </c>
@@ -3402,7 +4758,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
         <v>20</v>
       </c>
@@ -3410,7 +4766,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
         <v>31</v>
       </c>
@@ -3418,7 +4774,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>29</v>
       </c>
@@ -3426,7 +4782,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>18</v>
       </c>
@@ -3434,7 +4790,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="16" t="s">
         <v>59</v>
       </c>
@@ -3442,7 +4798,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
         <v>61</v>
       </c>
@@ -3450,7 +4806,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
         <v>23</v>
       </c>
@@ -3458,7 +4814,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
         <v>19</v>
       </c>
@@ -3466,7 +4822,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>64</v>
       </c>
@@ -3474,7 +4830,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>32</v>
       </c>
@@ -3482,7 +4838,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="s">
         <v>67</v>
       </c>
@@ -3490,7 +4846,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
         <v>16</v>
       </c>
@@ -3498,7 +4854,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
         <v>43</v>
       </c>
@@ -3506,7 +4862,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>36</v>
       </c>
@@ -3514,7 +4870,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
         <v>41</v>
       </c>
@@ -3522,7 +4878,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
         <v>45</v>
       </c>
@@ -3530,7 +4886,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="144" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
         <v>39</v>
       </c>
@@ -3538,7 +4894,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
         <v>47</v>
       </c>
@@ -3546,7 +4902,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
         <v>44</v>
       </c>
@@ -3554,7 +4910,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
         <v>30</v>
       </c>
@@ -3562,7 +4918,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
         <v>22</v>
       </c>
@@ -3570,7 +4926,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
         <v>48</v>
       </c>

</xml_diff>

<commit_message>
feat: implementar Pausa Turno Partido y correcciones de Sets
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Agosto.xlsx
+++ b/Cronograma de Tareas/Cronograma Agosto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B64BFF3-983D-4702-AD2B-0199540AD160}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12EFC43E-95B5-4475-9EFC-0A10AB51E5FA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{98BEDEB8-80D0-4DE0-A56F-770C1F3168B7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="98">
   <si>
     <t>Set 1 Mañana</t>
   </si>
@@ -553,17 +553,417 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="103">
+  <dxfs count="143">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1943,23 +2343,23 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="18"/>
+      <c r="C2" s="19"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="18"/>
-      <c r="H2" s="18" t="s">
+      <c r="F2" s="19"/>
+      <c r="H2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="18"/>
-      <c r="K2" s="18" t="s">
+      <c r="I2" s="19"/>
+      <c r="K2" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="L2" s="18"/>
+      <c r="L2" s="19"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
@@ -2191,10 +2591,10 @@
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="18"/>
+      <c r="C12" s="19"/>
       <c r="H12" s="6" t="s">
         <v>20</v>
       </c>
@@ -2216,10 +2616,10 @@
         <v>5</v>
       </c>
       <c r="D13" s="1"/>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="F13" s="18"/>
+      <c r="F13" s="19"/>
       <c r="H13" s="6" t="s">
         <v>23</v>
       </c>
@@ -2315,14 +2715,14 @@
       <c r="F17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H17" s="18" t="s">
+      <c r="H17" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="I17" s="18"/>
-      <c r="K17" s="18" t="s">
+      <c r="I17" s="19"/>
+      <c r="K17" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="L17" s="18"/>
+      <c r="L17" s="19"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
@@ -2429,10 +2829,10 @@
       <c r="C22" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E22" s="18" t="s">
+      <c r="E22" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="F22" s="18"/>
+      <c r="F22" s="19"/>
       <c r="H22" s="6" t="s">
         <v>13</v>
       </c>
@@ -2467,10 +2867,10 @@
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="C24" s="18"/>
+      <c r="C24" s="19"/>
       <c r="E24" s="6" t="s">
         <v>16</v>
       </c>
@@ -2609,14 +3009,14 @@
       <c r="C30" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="H30" s="18" t="s">
+      <c r="H30" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="I30" s="18"/>
-      <c r="K30" s="18" t="s">
+      <c r="I30" s="19"/>
+      <c r="K30" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="L30" s="18"/>
+      <c r="L30" s="19"/>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H31" s="3" t="s">
@@ -2727,114 +3127,114 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="IUqCyFrkbaZZs6cAzVH6yADvOKVmD+jfZ62LKfyUlQEBibwLjteZyT+2HPzW7vehSpQu4vmXZgLgmCKrwS2vqg==" saltValue="mjSDMFqxFcyaLmjD30rnTw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="102" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="142" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="101" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="141" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="100" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="140" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21">
-    <cfRule type="duplicateValues" dxfId="99" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="139" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26 E17:E18 B20">
-    <cfRule type="duplicateValues" dxfId="98" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="138" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27 B9">
-    <cfRule type="duplicateValues" dxfId="97" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="137" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="96" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="136" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="95" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="135" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="94" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="134" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="93" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="133" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10">
-    <cfRule type="duplicateValues" dxfId="92" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="132" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11">
-    <cfRule type="duplicateValues" dxfId="91" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="131" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E19 B10">
-    <cfRule type="duplicateValues" dxfId="90" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="130" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E27">
-    <cfRule type="duplicateValues" dxfId="89" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="129" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E28">
-    <cfRule type="duplicateValues" dxfId="88" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="128" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="87" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="127" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="86" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="126" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="85" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="125" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="84" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="124" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="83" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="123" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="82" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="122" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="81" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="121" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="80" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="120" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="79" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="119" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="78" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="118" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="77" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="117" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="76" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="116" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="75" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="115" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K23">
-    <cfRule type="duplicateValues" dxfId="74" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="114" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24:K25">
-    <cfRule type="duplicateValues" dxfId="73" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="113" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="72" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="112" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="71" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="111" priority="5"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2861,23 +3261,23 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="18"/>
+      <c r="C2" s="19"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="18"/>
-      <c r="H2" s="18" t="s">
+      <c r="F2" s="19"/>
+      <c r="H2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="18"/>
-      <c r="K2" s="18" t="s">
+      <c r="I2" s="19"/>
+      <c r="K2" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="L2" s="18"/>
+      <c r="L2" s="19"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
@@ -3083,10 +3483,10 @@
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="F11" s="18"/>
+      <c r="F11" s="19"/>
       <c r="H11" s="6" t="s">
         <v>90</v>
       </c>
@@ -3101,10 +3501,10 @@
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="18"/>
+      <c r="C12" s="19"/>
       <c r="E12" s="3" t="s">
         <v>6</v>
       </c>
@@ -3233,14 +3633,14 @@
       <c r="F17" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H17" s="18" t="s">
+      <c r="H17" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="I17" s="18"/>
-      <c r="K17" s="18" t="s">
+      <c r="I17" s="19"/>
+      <c r="K17" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="L17" s="18"/>
+      <c r="L17" s="19"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
@@ -3289,10 +3689,10 @@
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="E20" s="18" t="s">
+      <c r="E20" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="F20" s="18"/>
+      <c r="F20" s="19"/>
       <c r="H20" s="13" t="s">
         <v>19</v>
       </c>
@@ -3307,10 +3707,10 @@
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="C21" s="18"/>
+      <c r="C21" s="19"/>
       <c r="E21" s="3" t="s">
         <v>40</v>
       </c>
@@ -3515,14 +3915,14 @@
       <c r="C30" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H30" s="18" t="s">
+      <c r="H30" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="I30" s="18"/>
-      <c r="K30" s="18" t="s">
+      <c r="I30" s="19"/>
+      <c r="K30" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="L30" s="18"/>
+      <c r="L30" s="19"/>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="6" t="s">
@@ -3649,117 +4049,117 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="oIouQdWR80zfwrOgYg8mubgJdhcsB76Q9F8KDvzgM4ZHVaoaTdmBWqCttJGfgtEQSU1Z0+MmOBTlntxS+E5R6w==" saltValue="noKwfl3/0vFaNfkmv2IeLw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="70" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="110" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="69" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="109" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="68" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="108" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:B25">
-    <cfRule type="duplicateValues" dxfId="67" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="107" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26 B9">
-    <cfRule type="duplicateValues" dxfId="66" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="106" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27 B10">
-    <cfRule type="duplicateValues" dxfId="65" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="105" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
-    <cfRule type="duplicateValues" dxfId="64" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32">
-    <cfRule type="duplicateValues" dxfId="63" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="103" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="62" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="102" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="61" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="101" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="60" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="59" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="99" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16">
-    <cfRule type="duplicateValues" dxfId="58" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="98" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="57" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18">
-    <cfRule type="duplicateValues" dxfId="56" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
-    <cfRule type="duplicateValues" dxfId="55" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26">
-    <cfRule type="duplicateValues" dxfId="54" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="53" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="52" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="51" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="50" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H23">
-    <cfRule type="duplicateValues" dxfId="49" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24:H25">
-    <cfRule type="duplicateValues" dxfId="48" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="47" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="46" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="45" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="44" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="43" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="42" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K23">
-    <cfRule type="duplicateValues" dxfId="41" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24:K25">
-    <cfRule type="duplicateValues" dxfId="40" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="39" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="38" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="12"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3786,23 +4186,23 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="18"/>
+      <c r="C2" s="19"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="18"/>
-      <c r="H2" s="18" t="s">
+      <c r="F2" s="19"/>
+      <c r="H2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="18"/>
-      <c r="K2" s="18" t="s">
+      <c r="I2" s="19"/>
+      <c r="K2" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="L2" s="18"/>
+      <c r="L2" s="19"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
@@ -3871,13 +4271,13 @@
         <v>8</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>87</v>
+        <v>16</v>
       </c>
       <c r="I5" s="7" t="s">
         <v>8</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>87</v>
+        <v>16</v>
       </c>
       <c r="L5" s="7" t="s">
         <v>27</v>
@@ -3923,13 +4323,13 @@
         <v>8</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>88</v>
+        <v>21</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>8</v>
       </c>
       <c r="K7" s="8" t="s">
-        <v>88</v>
+        <v>21</v>
       </c>
       <c r="L7" s="7" t="s">
         <v>27</v>
@@ -3975,13 +4375,13 @@
         <v>8</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="I9" s="7" t="s">
         <v>8</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="L9" s="7" t="s">
         <v>27</v>
@@ -4001,13 +4401,13 @@
         <v>15</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>12</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L10" s="7" t="s">
         <v>11</v>
@@ -4027,13 +4427,13 @@
         <v>8</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>90</v>
+        <v>18</v>
       </c>
       <c r="I11" s="7" t="s">
         <v>8</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>90</v>
+        <v>18</v>
       </c>
       <c r="L11" s="7" t="s">
         <v>27</v>
@@ -4060,25 +4460,25 @@
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="18"/>
+      <c r="C13" s="19"/>
       <c r="D13" s="1"/>
       <c r="E13" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>8</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>91</v>
+        <v>23</v>
       </c>
       <c r="I13" s="7" t="s">
         <v>8</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>91</v>
+        <v>23</v>
       </c>
       <c r="L13" s="7" t="s">
         <v>27</v>
@@ -4093,7 +4493,7 @@
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>15</v>
@@ -4119,19 +4519,19 @@
         <v>28</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H15" s="9" t="s">
-        <v>92</v>
+      <c r="H15" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="I15" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="K15" s="9" t="s">
-        <v>92</v>
+      <c r="K15" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="L15" s="7" t="s">
         <v>27</v>
@@ -4144,12 +4544,7 @@
       <c r="C16" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E16" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="F16"/>
       <c r="G16" s="1"/>
       <c r="H16" s="8" t="s">
         <v>94</v>
@@ -4172,7 +4567,10 @@
       <c r="C17" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F17"/>
+      <c r="E17" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F17" s="19"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="6" t="s">
@@ -4181,18 +4579,20 @@
       <c r="C18" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E18" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="F18" s="18"/>
-      <c r="H18" s="18" t="s">
+      <c r="E18" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H18" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="I18" s="18"/>
-      <c r="K18" s="18" t="s">
+      <c r="I18" s="19"/>
+      <c r="K18" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="L18" s="18"/>
+      <c r="L18" s="19"/>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="8" t="s">
@@ -4201,11 +4601,11 @@
       <c r="C19" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>5</v>
+      <c r="E19" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>95</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>6</v>
@@ -4228,19 +4628,19 @@
         <v>28</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F20" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="H20" s="13" t="s">
-        <v>84</v>
+      <c r="H20" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="K20" s="13" t="s">
-        <v>84</v>
+      <c r="K20" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="L20" s="5" t="s">
         <v>17</v>
@@ -4248,18 +4648,18 @@
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="E21" s="6" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="F21" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="H21" s="13" t="s">
+      <c r="H21" s="6" t="s">
         <v>19</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="K21" s="13" t="s">
+      <c r="K21" s="6" t="s">
         <v>19</v>
       </c>
       <c r="L21" s="5" t="s">
@@ -4267,24 +4667,24 @@
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="C22" s="18"/>
+      <c r="C22" s="19"/>
       <c r="E22" s="6" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="H22" s="13" t="s">
-        <v>82</v>
+      <c r="H22" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="K22" s="13" t="s">
-        <v>82</v>
+      <c r="K22" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="L22" s="5" t="s">
         <v>17</v>
@@ -4298,19 +4698,19 @@
         <v>5</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F23" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="H23" s="13" t="s">
-        <v>7</v>
+      <c r="H23" s="6" t="s">
+        <v>13</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="K23" s="13" t="s">
-        <v>7</v>
+      <c r="K23" s="6" t="s">
+        <v>13</v>
       </c>
       <c r="L23" s="5" t="s">
         <v>28</v>
@@ -4323,40 +4723,34 @@
       <c r="C24" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E24" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="H24" s="13" t="s">
-        <v>23</v>
+      <c r="H24" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="K24" s="13" t="s">
-        <v>23</v>
+      <c r="K24" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="L24" s="5" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="25" spans="2:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="18" t="s">
         <v>46</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H25" s="13" t="s">
-        <v>83</v>
+      <c r="H25" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="K25" s="13" t="s">
-        <v>83</v>
+      <c r="K25" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="L25" s="5" t="s">
         <v>28</v>
@@ -4369,13 +4763,13 @@
       <c r="C26" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H26" s="13" t="s">
+      <c r="H26" s="6" t="s">
         <v>20</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="K26" s="13" t="s">
+      <c r="K26" s="6" t="s">
         <v>20</v>
       </c>
       <c r="L26" s="5" t="s">
@@ -4389,14 +4783,14 @@
       <c r="C27" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H27" s="13" t="s">
-        <v>24</v>
+      <c r="H27" s="6" t="s">
+        <v>23</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="K27" s="13" t="s">
-        <v>24</v>
+      <c r="K27" s="6" t="s">
+        <v>23</v>
       </c>
       <c r="L27" s="5" t="s">
         <v>28</v>
@@ -4409,13 +4803,13 @@
       <c r="C28" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H28" s="13" t="s">
+      <c r="H28" s="9" t="s">
         <v>29</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="K28" s="13" t="s">
+      <c r="K28" s="9" t="s">
         <v>29</v>
       </c>
       <c r="L28" s="5" t="s">
@@ -4429,14 +4823,14 @@
       <c r="C29" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H29" s="13" t="s">
-        <v>85</v>
+      <c r="H29" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="K29" s="13" t="s">
-        <v>85</v>
+      <c r="K29" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="L29" s="5" t="s">
         <v>28</v>
@@ -4479,14 +4873,14 @@
         <v>27</v>
       </c>
       <c r="D32"/>
-      <c r="H32" s="18" t="s">
+      <c r="H32" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="I32" s="18"/>
-      <c r="K32" s="18" t="s">
+      <c r="I32" s="19"/>
+      <c r="K32" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="L32" s="18"/>
+      <c r="L32" s="19"/>
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="6" t="s">
@@ -4603,123 +4997,129 @@
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="E18:F18"/>
     <mergeCell ref="H18:I18"/>
     <mergeCell ref="K18:L18"/>
+    <mergeCell ref="E17:F17"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="37" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="36" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="35" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="34"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B27 B24 B11">
+    <cfRule type="duplicateValues" dxfId="36" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28 B9">
-    <cfRule type="duplicateValues" dxfId="34" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="39"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29 B26">
+    <cfRule type="duplicateValues" dxfId="34" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31 B10">
-    <cfRule type="duplicateValues" dxfId="33" priority="36"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B29 B26">
-    <cfRule type="duplicateValues" dxfId="32" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="38"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B33">
+    <cfRule type="duplicateValues" dxfId="32" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="31" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="30" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="29" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="28" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10">
-    <cfRule type="duplicateValues" dxfId="27" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E13">
+    <cfRule type="duplicateValues" dxfId="26" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E14">
-    <cfRule type="duplicateValues" dxfId="26" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E15">
-    <cfRule type="duplicateValues" dxfId="25" priority="24"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E16">
-    <cfRule type="duplicateValues" dxfId="24" priority="12"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B33">
-    <cfRule type="duplicateValues" dxfId="23" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="20"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E22">
+    <cfRule type="duplicateValues" dxfId="23" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E23">
-    <cfRule type="duplicateValues" dxfId="22" priority="23"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E24">
-    <cfRule type="duplicateValues" dxfId="21" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="20" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="19" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="18" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="17" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H16">
-    <cfRule type="duplicateValues" dxfId="16" priority="4"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="15" priority="10"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H25:H26">
-    <cfRule type="duplicateValues" dxfId="14" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="18"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25">
+    <cfRule type="duplicateValues" dxfId="16" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H26">
+    <cfRule type="duplicateValues" dxfId="15" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H27">
+    <cfRule type="duplicateValues" dxfId="14" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H30">
-    <cfRule type="duplicateValues" dxfId="13" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H37">
-    <cfRule type="duplicateValues" dxfId="12" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H38">
-    <cfRule type="duplicateValues" dxfId="11" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="9" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="8" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="7" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K16">
-    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K24">
-    <cfRule type="duplicateValues" dxfId="5" priority="15"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K25:K26">
-    <cfRule type="duplicateValues" dxfId="4" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="17"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K25">
+    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K26">
+    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K27">
+    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K30">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K37">
-    <cfRule type="duplicateValues" dxfId="2" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K38">
-    <cfRule type="duplicateValues" dxfId="1" priority="17"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B27 B24 B11">
-    <cfRule type="duplicateValues" dxfId="0" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="23"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizacion de datos - mié 19/08/2026  7:58:35,78
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Agosto.xlsx
+++ b/Cronograma de Tareas/Cronograma Agosto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12EFC43E-95B5-4475-9EFC-0A10AB51E5FA}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2B7395A-8A89-420E-B862-9887EB8F844A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{98BEDEB8-80D0-4DE0-A56F-770C1F3168B7}"/>
   </bookViews>
@@ -563,387 +563,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="143">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="105">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3127,114 +2747,114 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="IUqCyFrkbaZZs6cAzVH6yADvOKVmD+jfZ62LKfyUlQEBibwLjteZyT+2HPzW7vehSpQu4vmXZgLgmCKrwS2vqg==" saltValue="mjSDMFqxFcyaLmjD30rnTw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B12:C12"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B12:C12"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="142" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="141" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="103" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="140" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="102" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21">
-    <cfRule type="duplicateValues" dxfId="139" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="101" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26 E17:E18 B20">
-    <cfRule type="duplicateValues" dxfId="138" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27 B9">
-    <cfRule type="duplicateValues" dxfId="137" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="99" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="136" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="98" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="135" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="134" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="133" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10">
-    <cfRule type="duplicateValues" dxfId="132" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11">
-    <cfRule type="duplicateValues" dxfId="131" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E19 B10">
-    <cfRule type="duplicateValues" dxfId="130" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E27">
-    <cfRule type="duplicateValues" dxfId="129" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E28">
-    <cfRule type="duplicateValues" dxfId="128" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="127" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="126" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="125" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="124" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="123" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="122" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="121" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="120" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="119" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="118" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="117" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="116" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="115" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K23">
-    <cfRule type="duplicateValues" dxfId="114" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24:K25">
-    <cfRule type="duplicateValues" dxfId="113" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="112" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="111" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="5"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4049,117 +3669,117 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="oIouQdWR80zfwrOgYg8mubgJdhcsB76Q9F8KDvzgM4ZHVaoaTdmBWqCttJGfgtEQSU1Z0+MmOBTlntxS+E5R6w==" saltValue="noKwfl3/0vFaNfkmv2IeLw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="110" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="109" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="108" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:B25">
-    <cfRule type="duplicateValues" dxfId="107" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26 B9">
-    <cfRule type="duplicateValues" dxfId="106" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27 B10">
-    <cfRule type="duplicateValues" dxfId="105" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
-    <cfRule type="duplicateValues" dxfId="104" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32">
-    <cfRule type="duplicateValues" dxfId="103" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="102" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="101" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="100" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="99" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16">
-    <cfRule type="duplicateValues" dxfId="98" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="97" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18">
-    <cfRule type="duplicateValues" dxfId="96" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
-    <cfRule type="duplicateValues" dxfId="95" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26">
-    <cfRule type="duplicateValues" dxfId="94" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="93" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="92" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="91" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="90" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H23">
-    <cfRule type="duplicateValues" dxfId="89" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24:H25">
-    <cfRule type="duplicateValues" dxfId="88" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="87" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="86" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="85" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="84" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="83" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="82" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K23">
-    <cfRule type="duplicateValues" dxfId="81" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24:K25">
-    <cfRule type="duplicateValues" dxfId="80" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="79" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="78" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="12"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4516,7 +4136,7 @@
         <v>16</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>48</v>
@@ -4565,7 +4185,7 @@
         <v>24</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="E17" s="19" t="s">
         <v>38</v>
@@ -4599,7 +4219,7 @@
         <v>21</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
Actualizacion de datos - mié 19/08/2026 12:15:09,34
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Agosto.xlsx
+++ b/Cronograma de Tareas/Cronograma Agosto.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2B7395A-8A89-420E-B862-9887EB8F844A}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D321A9A-A592-4E47-969F-F320A659843D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{98BEDEB8-80D0-4DE0-A56F-770C1F3168B7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{98BEDEB8-80D0-4DE0-A56F-770C1F3168B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 3 al 9 Ago" sheetId="4" r:id="rId1"/>
     <sheet name="Semana 2 - 10 al 16 Ago" sheetId="5" r:id="rId2"/>
     <sheet name="Semana 3 - 17 al 23 Ago" sheetId="6" r:id="rId3"/>
-    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId4"/>
+    <sheet name="Semana 4 - 24 al 30 Ago" sheetId="7" r:id="rId4"/>
+    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="969" uniqueCount="99">
   <si>
     <t>Set 1 Mañana</t>
   </si>
@@ -361,6 +362,9 @@
   </si>
   <si>
     <t>Revisión Calendarios</t>
+  </si>
+  <si>
+    <t>Apoyo con Deltas y GGR Negativo</t>
   </si>
 </sst>
 </file>
@@ -563,7 +567,427 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="105">
+  <dxfs count="147">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2747,114 +3171,114 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="IUqCyFrkbaZZs6cAzVH6yADvOKVmD+jfZ62LKfyUlQEBibwLjteZyT+2HPzW7vehSpQu4vmXZgLgmCKrwS2vqg==" saltValue="mjSDMFqxFcyaLmjD30rnTw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="104" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="146" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="103" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="145" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="102" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="144" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21">
-    <cfRule type="duplicateValues" dxfId="101" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="143" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26 E17:E18 B20">
-    <cfRule type="duplicateValues" dxfId="100" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="142" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27 B9">
-    <cfRule type="duplicateValues" dxfId="99" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="141" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="98" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="140" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="97" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="139" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="96" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="138" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="95" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="137" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10">
-    <cfRule type="duplicateValues" dxfId="94" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="136" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11">
-    <cfRule type="duplicateValues" dxfId="93" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="135" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E19 B10">
-    <cfRule type="duplicateValues" dxfId="92" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="134" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E27">
-    <cfRule type="duplicateValues" dxfId="91" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="133" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E28">
-    <cfRule type="duplicateValues" dxfId="90" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="132" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="89" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="131" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="88" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="130" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="87" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="129" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="86" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="128" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="85" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="127" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="84" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="126" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="83" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="125" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="82" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="124" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="81" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="123" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="80" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="122" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="79" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="121" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="78" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="120" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="77" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="119" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K23">
-    <cfRule type="duplicateValues" dxfId="76" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="118" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24:K25">
-    <cfRule type="duplicateValues" dxfId="75" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="117" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="74" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="116" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="73" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="115" priority="5"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3669,117 +4093,117 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="oIouQdWR80zfwrOgYg8mubgJdhcsB76Q9F8KDvzgM4ZHVaoaTdmBWqCttJGfgtEQSU1Z0+MmOBTlntxS+E5R6w==" saltValue="noKwfl3/0vFaNfkmv2IeLw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="72" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="114" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="71" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="113" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="70" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="112" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:B25">
-    <cfRule type="duplicateValues" dxfId="69" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="111" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26 B9">
-    <cfRule type="duplicateValues" dxfId="68" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="110" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27 B10">
-    <cfRule type="duplicateValues" dxfId="67" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="109" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
-    <cfRule type="duplicateValues" dxfId="66" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="108" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32">
-    <cfRule type="duplicateValues" dxfId="65" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="107" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="64" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="106" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="63" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="105" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="62" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="61" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="103" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16">
-    <cfRule type="duplicateValues" dxfId="60" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="102" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="59" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="101" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18">
-    <cfRule type="duplicateValues" dxfId="58" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
-    <cfRule type="duplicateValues" dxfId="57" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="99" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26">
-    <cfRule type="duplicateValues" dxfId="56" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="98" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="55" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="54" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="53" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="52" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H23">
-    <cfRule type="duplicateValues" dxfId="51" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24:H25">
-    <cfRule type="duplicateValues" dxfId="50" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="49" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="48" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="47" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="46" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="45" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="44" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K23">
-    <cfRule type="duplicateValues" dxfId="43" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24:K25">
-    <cfRule type="duplicateValues" dxfId="42" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="41" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="40" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="12"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4622,130 +5046,1125 @@
     <mergeCell ref="E17:F17"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="39" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="38" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="37" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="34"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27 B24 B11">
-    <cfRule type="duplicateValues" dxfId="36" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28 B9">
-    <cfRule type="duplicateValues" dxfId="35" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="39"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29 B26">
-    <cfRule type="duplicateValues" dxfId="34" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31 B10">
-    <cfRule type="duplicateValues" dxfId="33" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="38"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B33">
-    <cfRule type="duplicateValues" dxfId="32" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="31" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="30" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="29" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="28" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10">
-    <cfRule type="duplicateValues" dxfId="27" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E13">
-    <cfRule type="duplicateValues" dxfId="26" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E14">
-    <cfRule type="duplicateValues" dxfId="25" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E15">
-    <cfRule type="duplicateValues" dxfId="24" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E22">
-    <cfRule type="duplicateValues" dxfId="23" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E23">
-    <cfRule type="duplicateValues" dxfId="22" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="21" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="20" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="19" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="18" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H16">
-    <cfRule type="duplicateValues" dxfId="17" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="16" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="15" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H27">
-    <cfRule type="duplicateValues" dxfId="14" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H30">
-    <cfRule type="duplicateValues" dxfId="13" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H37">
-    <cfRule type="duplicateValues" dxfId="12" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H38">
-    <cfRule type="duplicateValues" dxfId="11" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="10" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="9" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="8" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="7" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K16">
-    <cfRule type="duplicateValues" dxfId="6" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K26">
-    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K27">
-    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K30">
-    <cfRule type="duplicateValues" dxfId="2" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K37">
-    <cfRule type="duplicateValues" dxfId="1" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K38">
-    <cfRule type="duplicateValues" dxfId="0" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="23"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A122ED22-5C30-4B4C-8699-855FFC6EDCA9}">
+  <dimension ref="B2:L41"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="3.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="54.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" style="2" customWidth="1"/>
+    <col min="5" max="5" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6" style="2" customWidth="1"/>
+    <col min="8" max="8" width="55" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.42578125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="55" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="15" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="19"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="19"/>
+      <c r="H2" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="I2" s="19"/>
+      <c r="K2" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="L2" s="19"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B9" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B10" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B11" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="E12" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B13" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="19"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="K14" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K15" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B16" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="J16" s="1"/>
+      <c r="K16" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B17" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="F17" s="19"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B18" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H18" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I18" s="19"/>
+      <c r="K18" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="L18" s="19"/>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B19" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="L19" s="12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="B20" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L20" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B21" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L21" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H22" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I22" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L22" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B23" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" s="19"/>
+      <c r="E23" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F23" s="19"/>
+      <c r="H23" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="L23" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B24" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B25" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L25" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="B26" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="L26" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B27" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L27" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B28" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K28" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="L28" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B29" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H29" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="K29" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="L29" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B30" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H30" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J30" s="1"/>
+      <c r="K30" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="L30" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B31" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B32" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32"/>
+      <c r="H32" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="I32" s="19"/>
+      <c r="K32" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="L32" s="19"/>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B33" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33"/>
+      <c r="H33" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K33" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="L33" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D34"/>
+      <c r="H34" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L34" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D35"/>
+      <c r="H35" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L35" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D36"/>
+      <c r="H36" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="L36" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D37"/>
+      <c r="H37" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I37" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L37" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D38"/>
+      <c r="H38" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I38" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="L38" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D39"/>
+    </row>
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D40"/>
+    </row>
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D41"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="E17:F17"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="duplicateValues" dxfId="41" priority="39"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7">
+    <cfRule type="duplicateValues" dxfId="40" priority="37"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8">
+    <cfRule type="duplicateValues" dxfId="39" priority="36"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29 B25 B11">
+    <cfRule type="duplicateValues" dxfId="38" priority="42"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B30 B9">
+    <cfRule type="duplicateValues" dxfId="37" priority="41"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B31 B27">
+    <cfRule type="duplicateValues" dxfId="36" priority="25"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B28 B10">
+    <cfRule type="duplicateValues" dxfId="35" priority="40"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B33">
+    <cfRule type="duplicateValues" dxfId="34" priority="26"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6">
+    <cfRule type="duplicateValues" dxfId="33" priority="35"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7">
+    <cfRule type="duplicateValues" dxfId="32" priority="34"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E8">
+    <cfRule type="duplicateValues" dxfId="31" priority="33"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9">
+    <cfRule type="duplicateValues" dxfId="30" priority="38"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E10">
+    <cfRule type="duplicateValues" dxfId="29" priority="23"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E13">
+    <cfRule type="duplicateValues" dxfId="28" priority="32"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E14">
+    <cfRule type="duplicateValues" dxfId="27" priority="31"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E15">
+    <cfRule type="duplicateValues" dxfId="26" priority="24"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4">
+    <cfRule type="duplicateValues" dxfId="25" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="duplicateValues" dxfId="24" priority="13"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12">
+    <cfRule type="duplicateValues" dxfId="23" priority="12"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="duplicateValues" dxfId="22" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H16">
+    <cfRule type="duplicateValues" dxfId="21" priority="22"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25">
+    <cfRule type="duplicateValues" dxfId="20" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H26">
+    <cfRule type="duplicateValues" dxfId="19" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H27">
+    <cfRule type="duplicateValues" dxfId="18" priority="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H30">
+    <cfRule type="duplicateValues" dxfId="17" priority="20"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H37">
+    <cfRule type="duplicateValues" dxfId="16" priority="30"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H38">
+    <cfRule type="duplicateValues" dxfId="15" priority="29"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4">
+    <cfRule type="duplicateValues" dxfId="14" priority="15"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11">
+    <cfRule type="duplicateValues" dxfId="13" priority="17"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12">
+    <cfRule type="duplicateValues" dxfId="12" priority="16"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K13">
+    <cfRule type="duplicateValues" dxfId="11" priority="18"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K16">
+    <cfRule type="duplicateValues" dxfId="10" priority="21"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K25">
+    <cfRule type="duplicateValues" dxfId="9" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K26">
+    <cfRule type="duplicateValues" dxfId="8" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K27">
+    <cfRule type="duplicateValues" dxfId="7" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K30">
+    <cfRule type="duplicateValues" dxfId="6" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K37">
+    <cfRule type="duplicateValues" dxfId="5" priority="28"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K38">
+    <cfRule type="duplicateValues" dxfId="4" priority="27"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E28">
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E29">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E19">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E21">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B623CE4C-92BF-4BB6-8978-4FC3B181F198}">
   <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="95.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Actualizacion de datos - mié 19/08/2026 12:24:26,87
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Agosto.xlsx
+++ b/Cronograma de Tareas/Cronograma Agosto.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="23" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D321A9A-A592-4E47-969F-F320A659843D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{98BEDEB8-80D0-4DE0-A56F-770C1F3168B7}"/>
+    <workbookView xWindow="28680" yWindow="5280" windowWidth="23280" windowHeight="12480" activeTab="3" xr2:uid="{98BEDEB8-80D0-4DE0-A56F-770C1F3168B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 3 al 9 Ago" sheetId="4" r:id="rId1"/>
@@ -3171,18 +3171,18 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="IUqCyFrkbaZZs6cAzVH6yADvOKVmD+jfZ62LKfyUlQEBibwLjteZyT+2HPzW7vehSpQu4vmXZgLgmCKrwS2vqg==" saltValue="mjSDMFqxFcyaLmjD30rnTw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B12:C12"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B12:C12"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="146" priority="29"/>
@@ -4093,18 +4093,18 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="oIouQdWR80zfwrOgYg8mubgJdhcsB76Q9F8KDvzgM4ZHVaoaTdmBWqCttJGfgtEQSU1Z0+MmOBTlntxS+E5R6w==" saltValue="noKwfl3/0vFaNfkmv2IeLw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="114" priority="30"/>
@@ -6021,18 +6021,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B13:C13"/>
     <mergeCell ref="H18:I18"/>
     <mergeCell ref="K18:L18"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="E23:F23"/>
     <mergeCell ref="H32:I32"/>
     <mergeCell ref="K32:L32"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="E17:F17"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="41" priority="39"/>
@@ -6043,17 +6043,17 @@
   <conditionalFormatting sqref="B8">
     <cfRule type="duplicateValues" dxfId="39" priority="36"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B28 B10">
+    <cfRule type="duplicateValues" dxfId="38" priority="40"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B29 B25 B11">
-    <cfRule type="duplicateValues" dxfId="38" priority="42"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="42"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30 B9">
-    <cfRule type="duplicateValues" dxfId="37" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="41"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31 B27">
-    <cfRule type="duplicateValues" dxfId="36" priority="25"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B28 B10">
-    <cfRule type="duplicateValues" dxfId="35" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B33">
     <cfRule type="duplicateValues" dxfId="34" priority="26"/>
@@ -6082,83 +6082,83 @@
   <conditionalFormatting sqref="E15">
     <cfRule type="duplicateValues" dxfId="26" priority="24"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E19">
+    <cfRule type="duplicateValues" dxfId="25" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E21">
+    <cfRule type="duplicateValues" dxfId="24" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E28">
+    <cfRule type="duplicateValues" dxfId="23" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E29">
+    <cfRule type="duplicateValues" dxfId="22" priority="3"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="25" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="24" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="23" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="22" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H16">
-    <cfRule type="duplicateValues" dxfId="21" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="20" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="19" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H27">
-    <cfRule type="duplicateValues" dxfId="18" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H30">
-    <cfRule type="duplicateValues" dxfId="17" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H37">
-    <cfRule type="duplicateValues" dxfId="16" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H38">
-    <cfRule type="duplicateValues" dxfId="15" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="14" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="13" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="12" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="11" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K16">
-    <cfRule type="duplicateValues" dxfId="10" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="duplicateValues" dxfId="9" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K26">
-    <cfRule type="duplicateValues" dxfId="8" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K27">
-    <cfRule type="duplicateValues" dxfId="7" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K30">
-    <cfRule type="duplicateValues" dxfId="6" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K37">
-    <cfRule type="duplicateValues" dxfId="5" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K38">
-    <cfRule type="duplicateValues" dxfId="4" priority="27"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E28">
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E29">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E19">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E21">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="27"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizacion de datos - mié 19/08/2026 14:21:24,96
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Agosto.xlsx
+++ b/Cronograma de Tareas/Cronograma Agosto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D321A9A-A592-4E47-969F-F320A659843D}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="8_{EFABAC76-4468-4D79-9781-2866BFFE3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18C4D957-9E38-4260-B13D-CCB691BFD708}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="5280" windowWidth="23280" windowHeight="12480" activeTab="3" xr2:uid="{98BEDEB8-80D0-4DE0-A56F-770C1F3168B7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{98BEDEB8-80D0-4DE0-A56F-770C1F3168B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 3 al 9 Ago" sheetId="4" r:id="rId1"/>
@@ -3171,18 +3171,18 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="IUqCyFrkbaZZs6cAzVH6yADvOKVmD+jfZ62LKfyUlQEBibwLjteZyT+2HPzW7vehSpQu4vmXZgLgmCKrwS2vqg==" saltValue="mjSDMFqxFcyaLmjD30rnTw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="146" priority="29"/>
@@ -4093,18 +4093,18 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="oIouQdWR80zfwrOgYg8mubgJdhcsB76Q9F8KDvzgM4ZHVaoaTdmBWqCttJGfgtEQSU1Z0+MmOBTlntxS+E5R6w==" saltValue="noKwfl3/0vFaNfkmv2IeLw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="114" priority="30"/>
@@ -4707,7 +4707,7 @@
         <v>19</v>
       </c>
       <c r="L21" s="5" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
@@ -4757,7 +4757,7 @@
         <v>13</v>
       </c>
       <c r="L23" s="5" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
@@ -4797,7 +4797,7 @@
         <v>18</v>
       </c>
       <c r="L25" s="5" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
@@ -4837,7 +4837,7 @@
         <v>23</v>
       </c>
       <c r="L27" s="5" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.25">
@@ -4877,7 +4877,7 @@
         <v>31</v>
       </c>
       <c r="L29" s="5" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.25">
@@ -4953,7 +4953,7 @@
         <v>16</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>95</v>
+        <v>28</v>
       </c>
       <c r="K34" s="6" t="s">
         <v>16</v>
@@ -4968,7 +4968,7 @@
         <v>19</v>
       </c>
       <c r="I35" s="5" t="s">
-        <v>95</v>
+        <v>28</v>
       </c>
       <c r="K35" s="6" t="s">
         <v>19</v>
@@ -4983,7 +4983,7 @@
         <v>44</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>95</v>
+        <v>28</v>
       </c>
       <c r="K36" s="6" t="s">
         <v>44</v>
@@ -4998,7 +4998,7 @@
         <v>29</v>
       </c>
       <c r="I37" s="5" t="s">
-        <v>95</v>
+        <v>28</v>
       </c>
       <c r="K37" s="6" t="s">
         <v>29</v>
@@ -5013,7 +5013,7 @@
         <v>31</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>95</v>
+        <v>28</v>
       </c>
       <c r="K38" s="6" t="s">
         <v>31</v>
@@ -6021,18 +6021,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="K32:L32"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="K32:L32"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="41" priority="39"/>

</xml_diff>